<commit_message>
Creacion de cedula sin EU
</commit_message>
<xml_diff>
--- a/src/assets/docs/plantilla_cedula.xlsx
+++ b/src/assets/docs/plantilla_cedula.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Mis Proyectos\PABS\interplazas\inter.ui\src\assets\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71A0BBCC-BA2D-4AEF-AB76-E6B2C79DDF19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72CDE06-75A3-4E5D-8783-E68DBC5E6186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-708" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="48">
   <si>
     <t>PROMOTORA FUTURA</t>
   </si>
@@ -252,9 +252,6 @@
   </si>
   <si>
     <t>{nombrePeriodo}</t>
-  </si>
-  <si>
-    <t>{FAVOR}</t>
   </si>
 </sst>
 </file>
@@ -1659,9 +1656,7 @@
       </c>
     </row>
     <row r="10" spans="1:14" s="7" customFormat="1" ht="12.75">
-      <c r="A10" s="27" t="s">
-        <v>48</v>
-      </c>
+      <c r="A10" s="27"/>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
       <c r="D10" s="27"/>

</xml_diff>